<commit_message>
ingress(kong) and rate limiting
</commit_message>
<xml_diff>
--- a/pov-terraform/Book1.xlsx
+++ b/pov-terraform/Book1.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10412"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/thant/Desktop/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/thant/cap_projects/pov-terraform/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{27231C71-0B8A-5D44-AB43-6575B168B7CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{784ED432-3426-CB43-B824-6C025DE501B5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="34560" windowHeight="21680" xr2:uid="{CBEB5DA0-E34F-4741-9D5A-6517805AB3B1}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="44" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="40">
   <si>
     <t>Component</t>
   </si>
@@ -153,6 +153,9 @@
   </si>
   <si>
     <t>Module Source for Module Version</t>
+  </si>
+  <si>
+    <t>AWS EKS</t>
   </si>
 </sst>
 </file>
@@ -429,7 +432,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -440,54 +443,54 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -496,9 +499,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="16" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -834,7 +834,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92487EA4-6155-A54F-AFCB-4F0F11D26BB5}">
-  <dimension ref="B4:F20"/>
+  <dimension ref="B4:G16"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="10.83203125" style="1"/>
@@ -843,196 +843,191 @@
     <col min="4" max="4" width="25.5" style="1" customWidth="1"/>
     <col min="5" max="5" width="50.33203125" style="1" customWidth="1"/>
     <col min="6" max="6" width="13.1640625" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="10.83203125" style="1"/>
+    <col min="7" max="7" width="16" style="1" customWidth="1"/>
+    <col min="8" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="4" spans="2:6" s="5" customFormat="1" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B4" s="18" t="s">
+    <row r="4" spans="2:7" s="4" customFormat="1" ht="40" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B4" s="15" t="s">
         <v>0</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="C4" s="15" t="s">
         <v>1</v>
       </c>
-      <c r="D4" s="18" t="s">
+      <c r="D4" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="E4" s="18" t="s">
+      <c r="E4" s="15" t="s">
         <v>38</v>
       </c>
-      <c r="F4" s="18" t="s">
+      <c r="F4" s="15" t="s">
         <v>34</v>
       </c>
-    </row>
-    <row r="5" spans="2:6" s="2" customFormat="1" ht="31" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B5" s="6" t="s">
+      <c r="G4" s="4" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="5" spans="2:7" s="2" customFormat="1" ht="31" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B5" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="7" t="s">
+      <c r="C5" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="8" t="s">
+      <c r="D5" s="7" t="s">
         <v>4</v>
       </c>
-      <c r="E5" s="7"/>
-      <c r="F5" s="19" t="s">
+      <c r="E5" s="6"/>
+      <c r="F5" s="16" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:6" s="2" customFormat="1" ht="31" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B6" s="9" t="s">
+    <row r="6" spans="2:7" s="2" customFormat="1" ht="31" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B6" s="8" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="10" t="s">
+      <c r="C6" s="9" t="s">
         <v>7</v>
       </c>
-      <c r="D6" s="11" t="s">
+      <c r="D6" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="E6" s="11" t="s">
+      <c r="E6" s="17" t="s">
         <v>36</v>
       </c>
       <c r="F6" s="20" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="2:6" s="2" customFormat="1" ht="31" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B7" s="12" t="s">
+    <row r="7" spans="2:7" s="2" customFormat="1" ht="31" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B7" s="10" t="s">
         <v>10</v>
       </c>
       <c r="C7" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
+      <c r="D7" s="19"/>
+      <c r="E7" s="19"/>
       <c r="F7" s="21"/>
     </row>
-    <row r="8" spans="2:6" s="2" customFormat="1" ht="31" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B8" s="12" t="s">
+    <row r="8" spans="2:7" s="2" customFormat="1" ht="31" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B8" s="10" t="s">
         <v>12</v>
       </c>
       <c r="C8" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="D8" s="4"/>
-      <c r="E8" s="4"/>
+      <c r="D8" s="19"/>
+      <c r="E8" s="19"/>
       <c r="F8" s="21"/>
     </row>
-    <row r="9" spans="2:6" s="2" customFormat="1" ht="31" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B9" s="12" t="s">
+    <row r="9" spans="2:7" s="2" customFormat="1" ht="31" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B9" s="10" t="s">
         <v>14</v>
       </c>
       <c r="C9" s="3" t="s">
         <v>15</v>
       </c>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
+      <c r="D9" s="19"/>
+      <c r="E9" s="19"/>
       <c r="F9" s="21"/>
     </row>
-    <row r="10" spans="2:6" s="2" customFormat="1" ht="31" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B10" s="12" t="s">
+    <row r="10" spans="2:7" s="2" customFormat="1" ht="31" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B10" s="10" t="s">
         <v>16</v>
       </c>
       <c r="C10" s="3" t="s">
         <v>17</v>
       </c>
-      <c r="D10" s="4"/>
-      <c r="E10" s="4"/>
+      <c r="D10" s="19"/>
+      <c r="E10" s="19"/>
       <c r="F10" s="21"/>
     </row>
-    <row r="11" spans="2:6" s="2" customFormat="1" ht="31" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B11" s="13" t="s">
+    <row r="11" spans="2:7" s="2" customFormat="1" ht="31" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B11" s="11" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="C11" s="12" t="s">
         <v>19</v>
       </c>
-      <c r="D11" s="15"/>
-      <c r="E11" s="15"/>
+      <c r="D11" s="18"/>
+      <c r="E11" s="18"/>
       <c r="F11" s="22"/>
     </row>
-    <row r="12" spans="2:6" s="2" customFormat="1" ht="31" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B12" s="9" t="s">
+    <row r="12" spans="2:7" s="2" customFormat="1" ht="31" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B12" s="8" t="s">
         <v>20</v>
       </c>
-      <c r="C12" s="10" t="s">
+      <c r="C12" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="D12" s="16" t="s">
+      <c r="D12" s="13" t="s">
         <v>22</v>
       </c>
-      <c r="E12" s="11" t="s">
+      <c r="E12" s="17" t="s">
         <v>37</v>
       </c>
       <c r="F12" s="20" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="13" spans="2:6" s="2" customFormat="1" ht="31" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B13" s="13" t="s">
+    <row r="13" spans="2:7" s="2" customFormat="1" ht="31" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B13" s="11" t="s">
         <v>23</v>
       </c>
-      <c r="C13" s="14" t="s">
+      <c r="C13" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="D13" s="17" t="s">
+      <c r="D13" s="14" t="s">
         <v>25</v>
       </c>
-      <c r="E13" s="15"/>
+      <c r="E13" s="18"/>
       <c r="F13" s="22"/>
     </row>
-    <row r="14" spans="2:6" s="2" customFormat="1" ht="31" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B14" s="6" t="s">
+    <row r="14" spans="2:7" s="2" customFormat="1" ht="31" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B14" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C14" s="7" t="s">
+      <c r="C14" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="D14" s="8" t="s">
+      <c r="D14" s="7" t="s">
         <v>27</v>
       </c>
-      <c r="E14" s="7"/>
-      <c r="F14" s="19" t="s">
+      <c r="E14" s="6"/>
+      <c r="F14" s="16" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="15" spans="2:6" s="2" customFormat="1" ht="31" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="B15" s="9" t="s">
+    <row r="15" spans="2:7" s="2" customFormat="1" ht="31" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="B15" s="8" t="s">
         <v>28</v>
       </c>
-      <c r="C15" s="10" t="s">
+      <c r="C15" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="D15" s="16" t="s">
+      <c r="D15" s="13" t="s">
         <v>30</v>
       </c>
-      <c r="E15" s="11" t="s">
+      <c r="E15" s="17" t="s">
         <v>35</v>
       </c>
       <c r="F15" s="20" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="16" spans="2:6" s="2" customFormat="1" ht="31" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="B16" s="13" t="s">
+    <row r="16" spans="2:7" s="2" customFormat="1" ht="31" customHeight="1" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="B16" s="11" t="s">
         <v>31</v>
       </c>
-      <c r="C16" s="14" t="s">
+      <c r="C16" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="D16" s="17" t="s">
+      <c r="D16" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="E16" s="15"/>
+      <c r="E16" s="18"/>
       <c r="F16" s="22"/>
-    </row>
-    <row r="18" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C18" s="23"/>
-    </row>
-    <row r="19" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C19" s="23"/>
-    </row>
-    <row r="20" spans="3:3" x14ac:dyDescent="0.2">
-      <c r="C20" s="23"/>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>